<commit_message>
Final_Records 2601/2502 갱신본 반영, Red and Black 인쇄본은 저장소에서 제외
</commit_message>
<xml_diff>
--- a/R/data/Final_Records_DS_2601_0620.xlsx
+++ b/R/data/Final_Records_DS_2601_0620.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kwlee/Documents/class202501/R/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{597E2DFA-7D4F-7449-8958-30BD86E37D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71461D56-38FE-774F-AB5C-AFBFD5F6768A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51160" yWindow="3340" windowWidth="44800" windowHeight="22740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="3320" windowWidth="44800" windowHeight="22740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="성적" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="200">
   <si>
     <t>이름</t>
   </si>
@@ -79,7 +79,7 @@
     <t>jts590@naver.com</t>
   </si>
   <si>
-    <t>B0</t>
+    <t>A0</t>
   </si>
   <si>
     <t>김낙현</t>
@@ -448,7 +448,7 @@
     <t>same1976@naver.com</t>
   </si>
   <si>
-    <t>C+</t>
+    <t>B+</t>
   </si>
   <si>
     <t>박성현</t>
@@ -578,9 +578,6 @@
   </si>
   <si>
     <t>ka2582@naver.com</t>
-  </si>
-  <si>
-    <t>C0</t>
   </si>
   <si>
     <t>반혁준</t>
@@ -1310,13 +1307,13 @@
         <v>19.7</v>
       </c>
       <c r="J8" s="2">
-        <v>9.17</v>
+        <v>10</v>
       </c>
       <c r="K8" s="2">
         <v>17.97</v>
       </c>
       <c r="L8" s="2">
-        <v>96.62</v>
+        <v>97.45</v>
       </c>
       <c r="M8" s="4" t="s">
         <v>25</v>
@@ -1925,16 +1922,16 @@
         <v>18.53</v>
       </c>
       <c r="J23" s="2">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="K23" s="2">
         <v>16.77</v>
       </c>
       <c r="L23" s="2">
-        <v>89.05</v>
+        <v>91.55</v>
       </c>
       <c r="M23" s="4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -1966,16 +1963,16 @@
         <v>17.32</v>
       </c>
       <c r="J24" s="2">
-        <v>7.5</v>
+        <v>9.17</v>
       </c>
       <c r="K24" s="2">
         <v>17.899999999999999</v>
       </c>
       <c r="L24" s="2">
-        <v>88.65</v>
+        <v>90.31</v>
       </c>
       <c r="M24" s="4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -2048,13 +2045,13 @@
         <v>17.82</v>
       </c>
       <c r="J26" s="2">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="K26" s="2">
         <v>16.87</v>
       </c>
       <c r="L26" s="2">
-        <v>86.25</v>
+        <v>88.75</v>
       </c>
       <c r="M26" s="4" t="s">
         <v>19</v>
@@ -2171,13 +2168,13 @@
         <v>18.899999999999999</v>
       </c>
       <c r="J29" s="2">
-        <v>8.33</v>
+        <v>10</v>
       </c>
       <c r="K29" s="2">
         <v>15.93</v>
       </c>
       <c r="L29" s="2">
-        <v>86.45</v>
+        <v>88.12</v>
       </c>
       <c r="M29" s="4" t="s">
         <v>19</v>
@@ -2212,13 +2209,13 @@
         <v>16.18</v>
       </c>
       <c r="J30" s="2">
-        <v>7.41</v>
+        <v>8.24</v>
       </c>
       <c r="K30" s="2">
         <v>10.07</v>
       </c>
       <c r="L30" s="2">
-        <v>66.69</v>
+        <v>67.52</v>
       </c>
       <c r="M30" s="4" t="s">
         <v>142</v>
@@ -2417,13 +2414,13 @@
         <v>18.54</v>
       </c>
       <c r="J35" s="2">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="K35" s="2">
         <v>17.7</v>
       </c>
       <c r="L35" s="2">
-        <v>93.1</v>
+        <v>95.6</v>
       </c>
       <c r="M35" s="4" t="s">
         <v>25</v>
@@ -2622,27 +2619,27 @@
         <v>7.16</v>
       </c>
       <c r="J40" s="2">
-        <v>6.67</v>
+        <v>7.5</v>
       </c>
       <c r="K40" s="2">
         <v>10.33</v>
       </c>
       <c r="L40" s="2">
-        <v>55.33</v>
+        <v>56.17</v>
       </c>
       <c r="M40" s="4" t="s">
-        <v>186</v>
+        <v>142</v>
       </c>
     </row>
     <row r="41" spans="1:13">
       <c r="A41" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="C41" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>189</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>16</v>
@@ -2651,7 +2648,7 @@
         <v>17</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G41" s="2">
         <v>20</v>
@@ -2677,22 +2674,22 @@
     </row>
     <row r="42" spans="1:13">
       <c r="A42" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="C42" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="D42" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E42" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D42" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E42" s="1" t="s">
+      <c r="F42" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="G42" s="2">
         <v>19</v>
@@ -2718,22 +2715,22 @@
     </row>
     <row r="43" spans="1:13">
       <c r="A43" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="C43" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="D43" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="D43" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>200</v>
       </c>
       <c r="G43" s="2">
         <v>20</v>
@@ -2758,6 +2755,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M44">
+    <sortCondition ref="C1:C44"/>
+  </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>